<commit_message>
Paradise Island stop-to-stop fares (29) from Jack's sheet v1
0039 adds Margaritaville and Carnival to every other stop. The website's
fares table now shows only Cruise Port trips, as its caption says; other
fares are quoted in the booking form. docs/fares-to-fill.xlsx regenerated
with the 91 pairs still to price.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fares-to-fill.xlsx
+++ b/docs/fares-to-fill.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Already priced" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -614,7 +614,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Already priced (from your first sheet) are on the 'Already priced' tab for reference.</t>
+          <t>Everything already live is on the 'Already priced' tab for reference.</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -669,12 +669,12 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C2" s="6" t="n"/>
@@ -684,12 +684,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -699,12 +699,12 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
@@ -714,12 +714,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
@@ -729,12 +729,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -744,12 +744,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C7" s="6" t="n"/>
@@ -759,12 +759,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C8" s="6" t="n"/>
@@ -774,12 +774,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
@@ -789,12 +789,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>
@@ -804,12 +804,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C11" s="6" t="n"/>
@@ -819,12 +819,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C12" s="6" t="n"/>
@@ -834,12 +834,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
@@ -849,12 +849,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
@@ -864,12 +864,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
@@ -879,12 +879,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
@@ -894,12 +894,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C17" s="6" t="n"/>
@@ -909,12 +909,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C18" s="6" t="n"/>
@@ -924,12 +924,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C19" s="6" t="n"/>
@@ -939,12 +939,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
@@ -954,12 +954,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
@@ -969,12 +969,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
@@ -984,12 +984,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
@@ -999,12 +999,12 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C24" s="6" t="n"/>
@@ -1014,12 +1014,12 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C25" s="6" t="n"/>
@@ -1029,12 +1029,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C26" s="6" t="n"/>
@@ -1044,12 +1044,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="C27" s="6" t="n"/>
@@ -1059,12 +1059,12 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C28" s="6" t="n"/>
@@ -1074,12 +1074,12 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C29" s="6" t="n"/>
@@ -1089,12 +1089,12 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C30" s="6" t="n"/>
@@ -1104,12 +1104,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C31" s="6" t="n"/>
@@ -1119,12 +1119,12 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C32" s="6" t="n"/>
@@ -1134,12 +1134,12 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C33" s="6" t="n"/>
@@ -1149,12 +1149,12 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C34" s="6" t="n"/>
@@ -1164,12 +1164,12 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C35" s="6" t="n"/>
@@ -1179,12 +1179,12 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C36" s="6" t="n"/>
@@ -1194,12 +1194,12 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C37" s="6" t="n"/>
@@ -1209,12 +1209,12 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C38" s="6" t="n"/>
@@ -1224,12 +1224,12 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C39" s="6" t="n"/>
@@ -1239,12 +1239,12 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C40" s="6" t="n"/>
@@ -1254,12 +1254,12 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C41" s="6" t="n"/>
@@ -1269,12 +1269,12 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C42" s="6" t="n"/>
@@ -1284,12 +1284,12 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C43" s="6" t="n"/>
@@ -1299,12 +1299,12 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C44" s="6" t="n"/>
@@ -1314,12 +1314,12 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C45" s="6" t="n"/>
@@ -1329,12 +1329,12 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C46" s="6" t="n"/>
@@ -1344,12 +1344,12 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C47" s="6" t="n"/>
@@ -1359,12 +1359,12 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C48" s="6" t="n"/>
@@ -1374,12 +1374,12 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C49" s="6" t="n"/>
@@ -1389,12 +1389,12 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C50" s="6" t="n"/>
@@ -1404,12 +1404,12 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C51" s="6" t="n"/>
@@ -1419,12 +1419,12 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C52" s="6" t="n"/>
@@ -1434,12 +1434,12 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C53" s="6" t="n"/>
@@ -1449,12 +1449,12 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C54" s="6" t="n"/>
@@ -1464,12 +1464,12 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C55" s="6" t="n"/>
@@ -1479,12 +1479,12 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C56" s="6" t="n"/>
@@ -1494,12 +1494,12 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C57" s="6" t="n"/>
@@ -1509,12 +1509,12 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C58" s="6" t="n"/>
@@ -1524,12 +1524,12 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C59" s="6" t="n"/>
@@ -1539,12 +1539,12 @@
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C60" s="6" t="n"/>
@@ -1554,12 +1554,12 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C61" s="6" t="n"/>
@@ -1569,12 +1569,12 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C62" s="6" t="n"/>
@@ -1584,12 +1584,12 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C63" s="6" t="n"/>
@@ -1599,12 +1599,12 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C64" s="6" t="n"/>
@@ -1614,12 +1614,12 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C65" s="6" t="n"/>
@@ -1629,12 +1629,12 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C66" s="6" t="n"/>
@@ -1644,12 +1644,12 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C67" s="6" t="n"/>
@@ -1659,12 +1659,12 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C68" s="6" t="n"/>
@@ -1674,12 +1674,12 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C69" s="6" t="n"/>
@@ -1689,12 +1689,12 @@
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C70" s="6" t="n"/>
@@ -1704,12 +1704,12 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C71" s="6" t="n"/>
@@ -1719,12 +1719,12 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C72" s="6" t="n"/>
@@ -1734,12 +1734,12 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C73" s="6" t="n"/>
@@ -1749,12 +1749,12 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C74" s="6" t="n"/>
@@ -1764,12 +1764,12 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C75" s="6" t="n"/>
@@ -1779,12 +1779,12 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C76" s="6" t="n"/>
@@ -1794,12 +1794,12 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C77" s="6" t="n"/>
@@ -1809,12 +1809,12 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C78" s="6" t="n"/>
@@ -1824,12 +1824,12 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C79" s="6" t="n"/>
@@ -1839,12 +1839,12 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C80" s="6" t="n"/>
@@ -1854,12 +1854,12 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C81" s="6" t="n"/>
@@ -1869,12 +1869,12 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C82" s="6" t="n"/>
@@ -1884,12 +1884,12 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C83" s="6" t="n"/>
@@ -1899,12 +1899,12 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C84" s="6" t="n"/>
@@ -1914,12 +1914,12 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C85" s="6" t="n"/>
@@ -1929,12 +1929,12 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C86" s="6" t="n"/>
@@ -1944,12 +1944,12 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C87" s="6" t="n"/>
@@ -1959,12 +1959,12 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C88" s="6" t="n"/>
@@ -1974,12 +1974,12 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C89" s="6" t="n"/>
@@ -1989,12 +1989,12 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C90" s="6" t="n"/>
@@ -2004,12 +2004,12 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C91" s="6" t="n"/>
@@ -2019,457 +2019,22 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C92" s="6" t="n"/>
       <c r="D92" s="6" t="n"/>
       <c r="E92" s="5" t="n"/>
     </row>
-    <row r="93">
-      <c r="A93" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B93" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="n"/>
-      <c r="D93" s="6" t="n"/>
-      <c r="E93" s="5" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B94" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="C94" s="6" t="n"/>
-      <c r="D94" s="6" t="n"/>
-      <c r="E94" s="5" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="n"/>
-      <c r="D95" s="6" t="n"/>
-      <c r="E95" s="5" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="n"/>
-      <c r="D96" s="6" t="n"/>
-      <c r="E96" s="5" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="n"/>
-      <c r="D97" s="6" t="n"/>
-      <c r="E97" s="5" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B98" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="n"/>
-      <c r="D98" s="6" t="n"/>
-      <c r="E98" s="5" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B99" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="n"/>
-      <c r="D99" s="6" t="n"/>
-      <c r="E99" s="5" t="n"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B100" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="n"/>
-      <c r="D100" s="6" t="n"/>
-      <c r="E100" s="5" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B101" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="C101" s="6" t="n"/>
-      <c r="D101" s="6" t="n"/>
-      <c r="E101" s="5" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B102" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="n"/>
-      <c r="D102" s="6" t="n"/>
-      <c r="E102" s="5" t="n"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B103" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C103" s="6" t="n"/>
-      <c r="D103" s="6" t="n"/>
-      <c r="E103" s="5" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C104" s="6" t="n"/>
-      <c r="D104" s="6" t="n"/>
-      <c r="E104" s="5" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="n"/>
-      <c r="D105" s="6" t="n"/>
-      <c r="E105" s="5" t="n"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B106" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="n"/>
-      <c r="D106" s="6" t="n"/>
-      <c r="E106" s="5" t="n"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B107" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C107" s="6" t="n"/>
-      <c r="D107" s="6" t="n"/>
-      <c r="E107" s="5" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B108" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C108" s="6" t="n"/>
-      <c r="D108" s="6" t="n"/>
-      <c r="E108" s="5" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B109" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C109" s="6" t="n"/>
-      <c r="D109" s="6" t="n"/>
-      <c r="E109" s="5" t="n"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B110" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C110" s="6" t="n"/>
-      <c r="D110" s="6" t="n"/>
-      <c r="E110" s="5" t="n"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B111" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="n"/>
-      <c r="D111" s="6" t="n"/>
-      <c r="E111" s="5" t="n"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B112" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C112" s="6" t="n"/>
-      <c r="D112" s="6" t="n"/>
-      <c r="E112" s="5" t="n"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C113" s="6" t="n"/>
-      <c r="D113" s="6" t="n"/>
-      <c r="E113" s="5" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C114" s="6" t="n"/>
-      <c r="D114" s="6" t="n"/>
-      <c r="E114" s="5" t="n"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C115" s="6" t="n"/>
-      <c r="D115" s="6" t="n"/>
-      <c r="E115" s="5" t="n"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B116" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C116" s="6" t="n"/>
-      <c r="D116" s="6" t="n"/>
-      <c r="E116" s="5" t="n"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C117" s="6" t="n"/>
-      <c r="D117" s="6" t="n"/>
-      <c r="E117" s="5" t="n"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B118" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C118" s="6" t="n"/>
-      <c r="D118" s="6" t="n"/>
-      <c r="E118" s="5" t="n"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="B119" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C119" s="6" t="n"/>
-      <c r="D119" s="6" t="n"/>
-      <c r="E119" s="5" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="B120" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C120" s="6" t="n"/>
-      <c r="D120" s="6" t="n"/>
-      <c r="E120" s="5" t="n"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="B121" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C121" s="6" t="n"/>
-      <c r="D121" s="6" t="n"/>
-      <c r="E121" s="5" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E121"/>
+  <autoFilter ref="A1:E92"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:D121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
+    <dataValidation sqref="C2:D92" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2483,7 +2048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2802,10 +2367,532 @@
         <v>70</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Source: your pickups.xlsx (5 Oct 2026). Live on the website now.</t>
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Señor Frog's</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Fort Montagu</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Señor Frog's</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D37" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Fort Montagu</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D39" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D45" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D46" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Source: your pickups.xlsx and fares-to-fill v1 (5 Oct 2026). All live now.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fares sheet v3: drop-off-only stops removed (55 pairs left)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fares-to-fill.xlsx
+++ b/docs/fares-to-fill.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Already priced" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -536,83 +536,90 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5. Leave a row blank and the office keeps quoting that trip by hand. Fill in only what you want.</t>
+          <t xml:space="preserve">   Pearl Island, Floating Bar and Blue Lagoon are drop-off only, so they have no rows here.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>6. Round trip blank but One way filled = round trip is charged as two one-ways.</t>
+          <t>5. Leave a row blank and the office keeps quoting that trip by hand. Fill in only what you want.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>7. Use the filter on the 'From' column to work through one stop at a time.</t>
+          <t>6. Round trip blank but One way filled = round trip is charged as two one-ways.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>7. Use the filter on the 'From' column to work through one stop at a time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>8. Send the file back and Coding loads every filled row into the live price list.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Example of a filled row (not in the sheet — just the format):</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>One way ($)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Round trip ($)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Señor Frog's</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C15" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D15" s="6" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Everything already live is on the 'Already priced' tab for reference.</t>
         </is>
@@ -629,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -669,12 +676,12 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C2" s="6" t="n"/>
@@ -684,12 +691,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -699,12 +706,12 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
@@ -714,12 +721,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
@@ -729,12 +736,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -744,12 +751,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C7" s="6" t="n"/>
@@ -759,12 +766,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C8" s="6" t="n"/>
@@ -774,12 +781,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
@@ -789,12 +796,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>
@@ -804,12 +811,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C11" s="6" t="n"/>
@@ -819,12 +826,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C12" s="6" t="n"/>
@@ -834,12 +841,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
@@ -849,12 +856,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
@@ -864,12 +871,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
@@ -879,12 +886,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
@@ -894,12 +901,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C17" s="6" t="n"/>
@@ -909,12 +916,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C18" s="6" t="n"/>
@@ -924,12 +931,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C19" s="6" t="n"/>
@@ -939,12 +946,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
@@ -954,12 +961,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
@@ -969,12 +976,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
@@ -984,12 +991,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
@@ -999,12 +1006,12 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C24" s="6" t="n"/>
@@ -1014,12 +1021,12 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C25" s="6" t="n"/>
@@ -1029,12 +1036,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C26" s="6" t="n"/>
@@ -1044,12 +1051,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C27" s="6" t="n"/>
@@ -1059,12 +1066,12 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C28" s="6" t="n"/>
@@ -1074,12 +1081,12 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C29" s="6" t="n"/>
@@ -1089,12 +1096,12 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C30" s="6" t="n"/>
@@ -1104,12 +1111,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C31" s="6" t="n"/>
@@ -1119,12 +1126,12 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C32" s="6" t="n"/>
@@ -1134,12 +1141,12 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C33" s="6" t="n"/>
@@ -1149,12 +1156,12 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C34" s="6" t="n"/>
@@ -1164,12 +1171,12 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C35" s="6" t="n"/>
@@ -1179,12 +1186,12 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C36" s="6" t="n"/>
@@ -1194,12 +1201,12 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C37" s="6" t="n"/>
@@ -1209,12 +1216,12 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C38" s="6" t="n"/>
@@ -1224,12 +1231,12 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C39" s="6" t="n"/>
@@ -1239,12 +1246,12 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C40" s="6" t="n"/>
@@ -1254,12 +1261,12 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C41" s="6" t="n"/>
@@ -1269,12 +1276,12 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C42" s="6" t="n"/>
@@ -1284,12 +1291,12 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C43" s="6" t="n"/>
@@ -1299,12 +1306,12 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C44" s="6" t="n"/>
@@ -1314,12 +1321,12 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C45" s="6" t="n"/>
@@ -1329,12 +1336,12 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C46" s="6" t="n"/>
@@ -1344,12 +1351,12 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C47" s="6" t="n"/>
@@ -1359,12 +1366,12 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C48" s="6" t="n"/>
@@ -1374,12 +1381,12 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C49" s="6" t="n"/>
@@ -1389,12 +1396,12 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C50" s="6" t="n"/>
@@ -1404,12 +1411,12 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C51" s="6" t="n"/>
@@ -1419,12 +1426,12 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C52" s="6" t="n"/>
@@ -1434,12 +1441,12 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C53" s="6" t="n"/>
@@ -1449,12 +1456,12 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C54" s="6" t="n"/>
@@ -1464,12 +1471,12 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C55" s="6" t="n"/>
@@ -1479,7 +1486,7 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
@@ -1491,550 +1498,10 @@
       <c r="D56" s="6" t="n"/>
       <c r="E56" s="5" t="n"/>
     </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="n"/>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="5" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="n"/>
-      <c r="D58" s="6" t="n"/>
-      <c r="E58" s="5" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="n"/>
-      <c r="D59" s="6" t="n"/>
-      <c r="E59" s="5" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="n"/>
-      <c r="D60" s="6" t="n"/>
-      <c r="E60" s="5" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C61" s="6" t="n"/>
-      <c r="D61" s="6" t="n"/>
-      <c r="E61" s="5" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="n"/>
-      <c r="D62" s="6" t="n"/>
-      <c r="E62" s="5" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="n"/>
-      <c r="D63" s="6" t="n"/>
-      <c r="E63" s="5" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>Poop Deck</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C64" s="6" t="n"/>
-      <c r="D64" s="6" t="n"/>
-      <c r="E64" s="5" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="n"/>
-      <c r="D65" s="6" t="n"/>
-      <c r="E65" s="5" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="n"/>
-      <c r="D66" s="6" t="n"/>
-      <c r="E66" s="5" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="n"/>
-      <c r="D67" s="6" t="n"/>
-      <c r="E67" s="5" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="n"/>
-      <c r="D68" s="6" t="n"/>
-      <c r="E68" s="5" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="n"/>
-      <c r="D69" s="6" t="n"/>
-      <c r="E69" s="5" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="n"/>
-      <c r="D70" s="6" t="n"/>
-      <c r="E70" s="5" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="n"/>
-      <c r="D71" s="6" t="n"/>
-      <c r="E71" s="5" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="n"/>
-      <c r="D72" s="6" t="n"/>
-      <c r="E72" s="5" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="n"/>
-      <c r="D73" s="6" t="n"/>
-      <c r="E73" s="5" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C74" s="6" t="n"/>
-      <c r="D74" s="6" t="n"/>
-      <c r="E74" s="5" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C75" s="6" t="n"/>
-      <c r="D75" s="6" t="n"/>
-      <c r="E75" s="5" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C76" s="6" t="n"/>
-      <c r="D76" s="6" t="n"/>
-      <c r="E76" s="5" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C77" s="6" t="n"/>
-      <c r="D77" s="6" t="n"/>
-      <c r="E77" s="5" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C78" s="6" t="n"/>
-      <c r="D78" s="6" t="n"/>
-      <c r="E78" s="5" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="n"/>
-      <c r="D79" s="6" t="n"/>
-      <c r="E79" s="5" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C80" s="6" t="n"/>
-      <c r="D80" s="6" t="n"/>
-      <c r="E80" s="5" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="n"/>
-      <c r="D81" s="6" t="n"/>
-      <c r="E81" s="5" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C82" s="6" t="n"/>
-      <c r="D82" s="6" t="n"/>
-      <c r="E82" s="5" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C83" s="6" t="n"/>
-      <c r="D83" s="6" t="n"/>
-      <c r="E83" s="5" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B84" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="n"/>
-      <c r="D84" s="6" t="n"/>
-      <c r="E84" s="5" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C85" s="6" t="n"/>
-      <c r="D85" s="6" t="n"/>
-      <c r="E85" s="5" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C86" s="6" t="n"/>
-      <c r="D86" s="6" t="n"/>
-      <c r="E86" s="5" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="n"/>
-      <c r="D87" s="6" t="n"/>
-      <c r="E87" s="5" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C88" s="6" t="n"/>
-      <c r="D88" s="6" t="n"/>
-      <c r="E88" s="5" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C89" s="6" t="n"/>
-      <c r="D89" s="6" t="n"/>
-      <c r="E89" s="5" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C90" s="6" t="n"/>
-      <c r="D90" s="6" t="n"/>
-      <c r="E90" s="5" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C91" s="6" t="n"/>
-      <c r="D91" s="6" t="n"/>
-      <c r="E91" s="5" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="B92" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="n"/>
-      <c r="D92" s="6" t="n"/>
-      <c r="E92" s="5" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E92"/>
+  <autoFilter ref="A1:E56"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:D92" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
+    <dataValidation sqref="C2:D56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Downtown stop-to-stop fares (27) from Jack's sheet v3
0041: Señor Frog's, Green Parrot and Poop Deck to the remaining stops.
0042: Poop Deck <-> Fort Montagu, held for a check and confirmed by Jack
($10 / $18). docs/fares-to-fill.xlsx regenerated with the 28 pairs left.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fares-to-fill.xlsx
+++ b/docs/fares-to-fill.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Already priced" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -676,12 +676,12 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C2" s="6" t="n"/>
@@ -691,12 +691,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -706,12 +706,12 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
@@ -721,12 +721,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
@@ -736,12 +736,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -751,12 +751,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C7" s="6" t="n"/>
@@ -766,12 +766,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C8" s="6" t="n"/>
@@ -781,12 +781,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
@@ -796,12 +796,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>
@@ -811,12 +811,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C11" s="6" t="n"/>
@@ -826,12 +826,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C12" s="6" t="n"/>
@@ -841,12 +841,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
@@ -856,12 +856,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
@@ -871,12 +871,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
@@ -886,12 +886,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
@@ -901,12 +901,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C17" s="6" t="n"/>
@@ -916,12 +916,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C18" s="6" t="n"/>
@@ -931,12 +931,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C19" s="6" t="n"/>
@@ -946,12 +946,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
@@ -961,12 +961,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
@@ -976,12 +976,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
@@ -991,12 +991,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
@@ -1006,12 +1006,12 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C24" s="6" t="n"/>
@@ -1021,12 +1021,12 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C25" s="6" t="n"/>
@@ -1036,12 +1036,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C26" s="6" t="n"/>
@@ -1051,7 +1051,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1066,7 +1066,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1081,427 +1081,22 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="5" t="n"/>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="5" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="5" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="5" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="5" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="5" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Fort Montagu</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="5" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="n"/>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" s="5" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="5" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="5" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="5" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="5" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Pigs Beach</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="5" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="6" t="n"/>
-      <c r="E42" s="5" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="5" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="n"/>
-      <c r="D44" s="6" t="n"/>
-      <c r="E44" s="5" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="n"/>
-      <c r="D45" s="6" t="n"/>
-      <c r="E45" s="5" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Rose Island – Goodies</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="n"/>
-      <c r="D46" s="6" t="n"/>
-      <c r="E46" s="5" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="n"/>
-      <c r="D47" s="6" t="n"/>
-      <c r="E47" s="5" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="n"/>
-      <c r="D48" s="6" t="n"/>
-      <c r="E48" s="5" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="n"/>
-      <c r="D49" s="6" t="n"/>
-      <c r="E49" s="5" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Junkanoo Beach</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="n"/>
-      <c r="D50" s="6" t="n"/>
-      <c r="E50" s="5" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="n"/>
-      <c r="D51" s="6" t="n"/>
-      <c r="E51" s="5" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="n"/>
-      <c r="D52" s="6" t="n"/>
-      <c r="E52" s="5" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="5" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="n"/>
-      <c r="D54" s="6" t="n"/>
-      <c r="E54" s="5" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Goodman's Bay</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="5" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>Breezes</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Baha Mar</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="n"/>
-      <c r="D56" s="6" t="n"/>
-      <c r="E56" s="5" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E56"/>
+  <autoFilter ref="A1:E29"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:D56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
+    <dataValidation sqref="C2:D29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1515,7 +1110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1855,55 +1450,55 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C19" s="11" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -1914,32 +1509,32 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24">
@@ -1950,32 +1545,32 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C25" s="11" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26">
@@ -1986,20 +1581,20 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C26" s="11" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -2022,14 +1617,14 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29">
@@ -2040,32 +1635,32 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31">
@@ -2076,205 +1671,205 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C31" s="11" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C32" s="11" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D34" s="11" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D36" s="11" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C37" s="11" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C38" s="11" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D38" s="11" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C39" s="11" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C40" s="11" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D40" s="11" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C41" s="11" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C42" s="11" t="n">
@@ -2287,43 +1882,43 @@
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C43" s="11" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C44" s="11" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D44" s="11" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -2341,23 +1936,509 @@
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D46" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D47" s="11" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
           <t>Paradise Island – Carnival</t>
         </is>
       </c>
-      <c r="B46" s="10" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D50" s="11" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D52" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D53" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D54" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>Baha Mar</t>
         </is>
       </c>
-      <c r="C46" s="11" t="n">
+      <c r="C55" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="D55" s="11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Señor Frog's</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D56" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>Green Parrot</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D57" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D58" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D59" s="11" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D60" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D61" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>Fort Montagu</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D62" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D63" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D64" s="11" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D65" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D46" s="11" t="n">
+      <c r="D66" s="11" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D67" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D68" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D69" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="D70" s="11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D71" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D72" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D73" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
         <is>
           <t>Source: your pickups.xlsx and fares-to-fill v1 (5 Oct 2026). All live now.</t>
         </is>

</xml_diff>

<commit_message>
Fares sheet: trips to the drop-off-only stops (39)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fares-to-fill.xlsx
+++ b/docs/fares-to-fill.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Already priced" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fares to fill'!$A$1:$E$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -498,7 +498,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Paradise Sea Express — fares between your 17 stops</t>
+          <t>Paradise Sea Express — fares to the drop-off-only stops</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1. Go to the 'Fares to fill' tab. Each row is one trip between two stops.</t>
+          <t>1. Go to the 'Fares to fill' tab. Each row is a trip from a pickup stop (From) to a drop-off-only stop (To).</t>
         </is>
       </c>
     </row>
@@ -529,97 +529,90 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4. A trip costs the same in both directions, so each pair is listed once.</t>
+          <t>4. Round trip = out to the drop-off stop and back to where they started.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pearl Island, Floating Bar, Blue Lagoon, Pigs Beach and Rose Island – Goodies are drop-off only, so they have no rows here.</t>
+          <t>5. Leave a row blank and the office keeps quoting that trip by hand. Fill in only what you want.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5. Leave a row blank and the office keeps quoting that trip by hand. Fill in only what you want.</t>
+          <t>6. Round trip blank but One way filled = round trip is charged as two one-ways.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>6. Round trip blank but One way filled = round trip is charged as two one-ways.</t>
+          <t>7. Use the filter on the 'From' column to work through one stop at a time.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>7. Use the filter on the 'From' column to work through one stop at a time.</t>
+          <t>8. Send the file back and Coding loads every filled row into the live price list.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>8. Send the file back and Coding loads every filled row into the live price list.</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Example of a filled row (not in the sheet — just the format):</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Example of a filled row (not in the sheet — just the format):</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>One way ($)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Round trip ($)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>From</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>To</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>One way ($)</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Round trip ($)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Paradise Island – Margaritaville</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Señor Frog's</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Everything already live is on the 'Already priced' tab for reference.</t>
         </is>
@@ -636,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -676,12 +669,12 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C2" s="6" t="n"/>
@@ -691,12 +684,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -706,12 +699,12 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
@@ -721,12 +714,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
@@ -736,12 +729,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
@@ -751,12 +744,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C7" s="6" t="n"/>
@@ -766,12 +759,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C8" s="6" t="n"/>
@@ -781,12 +774,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
@@ -796,12 +789,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C10" s="6" t="n"/>
@@ -811,12 +804,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C11" s="6" t="n"/>
@@ -826,12 +819,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C12" s="6" t="n"/>
@@ -841,12 +834,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
@@ -856,12 +849,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
@@ -871,12 +864,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
@@ -886,22 +879,382 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="5" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="5" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Pearl Island</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="5" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Floating Bar</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="5" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="5" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E16"/>
+  <autoFilter ref="A1:E40"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:D16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
+    <dataValidation sqref="C2:D40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Price" error="Enter a dollar amount above 0, or leave it blank." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -915,7 +1268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:D90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1237,12 +1590,12 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
@@ -1255,12 +1608,12 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Paradise Island – Carnival</t>
         </is>
       </c>
       <c r="C19" s="11" t="n">
@@ -1273,91 +1626,91 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
@@ -1368,14 +1721,14 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C25" s="11" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26">
@@ -1386,50 +1739,50 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C26" s="11" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
@@ -1440,14 +1793,14 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30">
@@ -1458,122 +1811,122 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C31" s="11" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
+          <t>Paradise Island – Margaritaville</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
           <t>Señor Frog's</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Arawak Cay / Fish Fry</t>
-        </is>
-      </c>
       <c r="C32" s="11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D34" s="11" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>70</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D36" s="11" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37">
@@ -1584,14 +1937,14 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C37" s="11" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38">
@@ -1602,97 +1955,97 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C38" s="11" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="D38" s="11" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C39" s="11" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C40" s="11" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D40" s="11" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C41" s="11" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C42" s="11" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D42" s="11" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C43" s="11" t="n">
@@ -1705,7 +2058,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -1723,7 +2076,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -1741,43 +2094,43 @@
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C46" s="11" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D46" s="11" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C47" s="11" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D47" s="11" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Margaritaville</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -1795,48 +2148,48 @@
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C49" s="11" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D49" s="11" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Pearl Island</t>
+          <t>Poop Deck</t>
         </is>
       </c>
       <c r="C50" s="11" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D50" s="11" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Floating Bar</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C51" s="11" t="n">
@@ -1849,37 +2202,37 @@
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C52" s="11" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D52" s="11" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Blue Lagoon</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C53" s="11" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D53" s="11" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="54">
@@ -1890,218 +2243,218 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Fort Montagu</t>
         </is>
       </c>
       <c r="C54" s="11" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D54" s="11" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C55" s="11" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="D55" s="11" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Señor Frog's</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="C56" s="11" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D56" s="11" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Green Parrot</t>
+          <t>Pigs Beach</t>
         </is>
       </c>
       <c r="C57" s="11" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D57" s="11" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Rose Island – Goodies</t>
         </is>
       </c>
       <c r="C58" s="11" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D58" s="11" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="C59" s="11" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="D59" s="11" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Goodman's Bay</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C60" s="11" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D60" s="11" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Breezes</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C61" s="11" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D61" s="11" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Paradise Island – Margaritaville</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Fort Montagu</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C62" s="11" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="D62" s="11" t="n">
-        <v>28</v>
+        <v>70</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Pigs Beach</t>
+          <t>Junkanoo Beach</t>
         </is>
       </c>
       <c r="C63" s="11" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D63" s="11" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Paradise Island – Carnival</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Pearl Island</t>
         </is>
       </c>
       <c r="C64" s="11" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D64" s="11" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Rose Island – Goodies</t>
+          <t>Arawak Cay / Fish Fry</t>
         </is>
       </c>
       <c r="C65" s="11" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="D65" s="11" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -2124,20 +2477,20 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Junkanoo Beach</t>
+          <t>Floating Bar</t>
         </is>
       </c>
       <c r="C67" s="11" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D67" s="11" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
@@ -2160,50 +2513,50 @@
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Arawak Cay / Fish Fry</t>
+          <t>Blue Lagoon</t>
         </is>
       </c>
       <c r="C69" s="11" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D69" s="11" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>Poop Deck</t>
+          <t>Paradise Island – Carnival</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Baha Mar</t>
+          <t>Señor Frog's</t>
         </is>
       </c>
       <c r="C70" s="11" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="D70" s="11" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>Paradise Island – Carnival</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Goodman's Bay</t>
+          <t>Baha Mar</t>
         </is>
       </c>
       <c r="C71" s="11" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="72">
@@ -2214,36 +2567,306 @@
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Breezes</t>
+          <t>Green Parrot</t>
         </is>
       </c>
       <c r="C72" s="11" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D72" s="11" t="n">
-        <v>70</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D73" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
           <t>Paradise Island – Carnival</t>
         </is>
       </c>
-      <c r="B73" s="10" t="inlineStr">
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D74" s="11" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D75" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>Fort Montagu</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D76" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D77" s="11" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>Pigs Beach</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D78" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D79" s="11" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="C80" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D80" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B81" s="10" t="inlineStr">
+        <is>
+          <t>Rose Island – Goodies</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D81" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>Junkanoo Beach</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D82" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D83" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>Poop Deck</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
         <is>
           <t>Baha Mar</t>
         </is>
       </c>
-      <c r="C73" s="11" t="n">
+      <c r="C84" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="D84" s="11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>Arawak Cay / Fish Fry</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D85" s="11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>Goodman's Bay</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>Breezes</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="D73" s="11" t="n">
+      <c r="D87" s="11" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="7" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="10" t="inlineStr">
+        <is>
+          <t>Paradise Island – Carnival</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>Baha Mar</t>
+        </is>
+      </c>
+      <c r="C88" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>Source: your pickups.xlsx and fares-to-fill v1 (5 Oct 2026). All live now.</t>
         </is>

</xml_diff>